<commit_message>
SOUL S: final consistency fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01Ck8guzeJBknbgPsaU2FiFA
</commit_message>
<xml_diff>
--- a/micul-smecher/docs/factory/SOUL-fabrica-model.xlsx
+++ b/micul-smecher/docs/factory/SOUL-fabrica-model.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Citește-mă" sheetId="1" state="visible" r:id="rId3"/>
@@ -381,7 +381,7 @@
     <t xml:space="preserve">cod</t>
   </si>
   <si>
-    <t xml:space="preserve">02-MANUFACTURING §11: PCB custom de la ~1k buc. La 100 buc. NRE-ul PCB (~$15–30k) nu se justifică → placa Waveshare [estimare]. Atenție: cu placa Waveshare corpul e S-P0 (25,65 mm, 500 mAh; docs/12 §2.3), nu produsul de 23 mm</t>
+    <t xml:space="preserve">02-MANUFACTURING §11: PCB custom de la ~1k buc. La 100 buc. NRE-ul PCB (~$15–30k) nu se justifică → placa Waveshare [estimare]. Atenție: cu placa Waveshare corpul e S-P0 (25,65 mm, LiPo 503030 ~450 mAh [estimare]; docs/12 §2.3), nu produsul de 23 mm</t>
   </si>
   <si>
     <t xml:space="preserve">pcba_sel</t>
@@ -576,10 +576,10 @@
     <t xml:space="preserve">battery_usd</t>
   </si>
   <si>
-    <t xml:space="preserve">Celulă LiPo 603040 750 mAh cu PCM (la 100 buc. cu placa Waveshare: 503035 500 mAh, S-P0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/12 §3.1: 503035 ≈ 3,00 € la 100 (S-P0); 603040 $1,5 la 1.000 [estimare]; listarea A&amp;S Power 603040 750 mAh (HKTDC). Cere UN38.3 + IEC 62133.</t>
+    <t xml:space="preserve">Celulă LiPo 603040 750 mAh cu PCM (la 100 buc. cu placa Waveshare: 503030 ~450 mAh, S-P0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/12 §3.1: 503030 ≈ 3,00 € la 100 (S-P0) [estimare]; 603040 $1,5 la 1.000 [estimare]; listarea A&amp;S Power 603040 750 mAh (HKTDC). Cere UN38.3 + IEC 62133.</t>
   </si>
   <si>
     <t xml:space="preserve">speaker_eur</t>
@@ -777,7 +777,7 @@
     <t xml:space="preserve">€/set</t>
   </si>
   <si>
-    <t xml:space="preserve">[estimare] = valorile M (85 / 35 / 27 / 22) × 0,65, factorul carcasei S externe din docs/12 §3.1 (suprafață × 0,50, semifabricat × 0,40, taxe fixe); Vault: S @25 = 92 €/set cu finisaj (BOM P0-12); 1k China $25–45/set pentru S (02-MANUFACTURING §11); curba PREMSA 6061 ~100×70×40: $118 @1 / $61 @25 / $54 @100 (https://premsaindustries.com/en/aluminum-machining). La ≥10k dosarul trece pe ambutisare 5052 (nemodelat).</t>
+    <t xml:space="preserve">[estimare] = valorile M (85 / 35 / 27 / 22) × 0,65, factorul carcasei S externe din docs/12 §3.1 și size-s.json cnc.external_shell_factor_vs_M, același în modelul de obiectiv al campaniei (suprafață × 0,50, semifabricat × 0,40, taxe fixe); Vault: S @25 = 92 €/set cu finisaj (BOM P0-12); 1k China $25–45/set pentru S (02-MANUFACTURING §11); curba PREMSA 6061 ~100×70×40: $118 @1 / $61 @25 / $54 @100 (https://premsaindustries.com/en/aluminum-machining). La ≥10k dosarul trece pe ambutisare 5052 (nemodelat).</t>
   </si>
   <si>
     <t xml:space="preserve">blast_buy_eur</t>
@@ -1707,7 +1707,7 @@
     <t xml:space="preserve">batt</t>
   </si>
   <si>
-    <t xml:space="preserve">Baterie LiPo 750 mAh (500 mAh la S-P0)</t>
+    <t xml:space="preserve">Baterie LiPo 750 mAh (~450 mAh la S-P0)</t>
   </si>
   <si>
     <t xml:space="preserve">glass</t>
@@ -2728,19 +2728,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; buc/an&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;;\-#,##0.00&quot; €&quot;;\-"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; €&quot;;\-#,##0&quot; €&quot;;\-"/>
     <numFmt numFmtId="168" formatCode="#,##0;\-#,##0;\-"/>
     <numFmt numFmtId="169" formatCode="#,##0.0;\-#,##0.0;\-"/>
-    <numFmt numFmtId="170" formatCode="#,##0.00;\-#,##0.00;\-"/>
-    <numFmt numFmtId="171" formatCode="0.0%;\-0.0%;\-"/>
-    <numFmt numFmtId="172" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="173" formatCode="0.0000"/>
-    <numFmt numFmtId="174" formatCode="#,##0&quot; lei&quot;"/>
-    <numFmt numFmtId="175" formatCode="#,##0&quot; buc&quot;"/>
+    <numFmt numFmtId="170" formatCode="General"/>
+    <numFmt numFmtId="171" formatCode="#,##0.00;\-#,##0.00;\-"/>
+    <numFmt numFmtId="172" formatCode="0.0%;\-0.0%;\-"/>
+    <numFmt numFmtId="173" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="0.0000"/>
+    <numFmt numFmtId="175" formatCode="#,##0&quot; lei&quot;"/>
+    <numFmt numFmtId="176" formatCode="#,##0&quot; buc&quot;"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -2967,7 +2968,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2979,7 +2980,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2991,7 +2992,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3003,7 +3004,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3011,7 +3012,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3023,7 +3024,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3031,11 +3032,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3055,7 +3056,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3091,7 +3092,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5895,7 +5896,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="17" t="s">
         <v>247</v>
       </c>

</xml_diff>